<commit_message>
feat(config): auto-detect stale mapping configs
</commit_message>
<xml_diff>
--- a/test_data/VNPAY_2024-07-08.xlsx
+++ b/test_data/VNPAY_2024-07-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>500219</v>
+        <v>50019</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024-07-08 06:50:56</t>
+          <t>2024-07-08 15:03:28</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1000351</v>
+        <v>300903</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2024-07-08 20:47:24</t>
+          <t>2024-07-08 21:17:08</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>500114</v>
+        <v>150340</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2024-07-08 04:51:44</t>
+          <t>2024-07-08 20:21:32</t>
         </is>
       </c>
     </row>
@@ -530,16 +530,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>100155</v>
+        <v>500532</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024-07-08 02:57:23</t>
+          <t>2024-07-08 01:02:41</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>100291</v>
+        <v>100784</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -564,7 +564,132 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024-07-08 16:49:20</t>
+          <t>2024-07-08 08:30:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VNP000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VNPY240708TXN000006</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>300538</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2024-07-08 03:22:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VNP000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VNPY240708TXN000007</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>300388</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2024-07-08 07:02:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VNP000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>VNPY240708TXN000008</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>300441</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2024-07-08 06:16:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VNP000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>VNPY240708TXN000009</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>100292</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2024-07-08 06:37:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VNP000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>VNPY240708TXN000010</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5000677</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2024-07-08 22:06:43</t>
         </is>
       </c>
     </row>

</xml_diff>